<commit_message>
feat: 技能效果系统完善 —— ApplySkillEffects 按 TargetType 分派 + MP 追踪 + 治疗技能
- UGA_DataDriven 新增 ApplySkillEffects：根据 TargetType (Self/Enemy/Area) 分派 GE，
  近战技能 (有 AttackMontage) 的 Enemy 效果留给武器碰撞 OnAttackHit 判定，
  非近战技能立即通过 Overlap 扫描寻找目标
- UGA_DataDriven 补充 CheckCost/ApplyCost/CheckCooldown/ApplyCooldown 全覆盖，
  冷却用 DynamicGrantedTags 实现，消耗按 CostType 动态创建 Instant GE
- UAttributeSet_Base 新增 MP 变化追踪 (OnMPChanged/OnRep_MP/MPBeforeAttributeChange)
- ABaseCharacter 添加 HP/MP 屏幕调试打印，MP delegate 绑定与广播
- 新增 Healing 技能配置和 Healing_RestoreHP 效果行 (Effect.Heal→负值 IncomingDamage)
- GameplayTags 扩展：Skill 输入、Cooldown、Passive、Trigger、Attr/Cost/Target 标签
- UAbilitySet 授予时写入 InputTag 到 DynamicAbilityTags
- AInGamePlayerController 重构为 InputConfig DataAsset 驱动技能输入绑定

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Config/Data/DT_SkillConfig.xlsx
+++ b/Content/Config/Data/DT_SkillConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\UnrealEngine\UEProject\FrontendUI\Content\Config\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A62305-FB5D-4104-BB8D-83CB2CA9FDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0E5A01-A49A-48EA-A6B5-1BD4D3025536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{2C778187-25A6-4551-9EB6-C2C1EAC8F6EE}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Name</t>
   </si>
@@ -93,6 +93,34 @@
   </si>
   <si>
     <t>/Script/Engine.AnimMontage'/Game/Gameplay/Player/Montage/MA_Melee.MA_Melee'</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>NSLOCTEXT(,,重攻击)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Healing</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>(Tag=Cost.MP)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>(Tag=Skill.Healing)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>(Tags=Skill.Healing)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>NSLOCTEXT(,,Heal)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Script/Engine.Texture2D'/Game/Assets/UI/Icons/HealthRegen.HealthRegen'</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1065,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A055F7F9-2A81-49D4-B1E3-5F3D418503E1}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.5" customWidth="1"/>
@@ -1074,7 +1102,8 @@
     <col min="4" max="4" width="24.33203125" customWidth="1"/>
     <col min="6" max="6" width="17.9140625" customWidth="1"/>
     <col min="7" max="7" width="22.1640625" customWidth="1"/>
-    <col min="11" max="11" width="52.9140625" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="27.83203125" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
     <col min="13" max="13" width="17.9140625" customWidth="1"/>
   </cols>
@@ -1166,7 +1195,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -1190,11 +1219,50 @@
         <v>18</v>
       </c>
       <c r="M3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4">
+        <v>15</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="L4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>